<commit_message>
Fix video mobile scaling and update whitelist API route
</commit_message>
<xml_diff>
--- a/whitelist.xlsx
+++ b/whitelist.xlsx
@@ -1,50 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C3E106-5B85-42E3-8A4C-261646C6D698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Whitelist" state="visible" r:id="rId4"/>
+    <sheet name="Whitelist" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>0xddc45a2286903bca89dbe8b3176020bcff7a6c6d</t>
-  </si>
-  <si>
-    <t>connected</t>
-  </si>
-  <si>
-    <t>2026-08-19T14:30:11.753Z</t>
-  </si>
-  <si>
-    <t>0xddc45a2286903bca89dbe8b3176020bcff7a6c65</t>
-  </si>
-  <si>
-    <t>manual</t>
-  </si>
-  <si>
-    <t>2026-08-19T14:30:30.157Z</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -407,9 +389,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.44140625" customWidth="1"/>
   </cols>
@@ -419,28 +401,8 @@
     <row r="3" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="13" x14ac:dyDescent="0.25"/>
+    <row r="14" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>